<commit_message>
feat: add visual-review alt coverage for all local images
</commit_message>
<xml_diff>
--- a/docs/Sunlit_Image_Alt_Manual_Review.xlsx
+++ b/docs/Sunlit_Image_Alt_Manual_Review.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待人工复核 (56)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="视觉识别补充 alt (56)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已继承 WordPress alt (138)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文章图片 (18)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'待人工复核 (56)'!$A$1:$L$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'视觉识别补充 alt (56)'!$A$1:$L$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'已继承 WordPress alt (138)'!$A$1:$L$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'文章图片 (18)'!$A$1:$L$19</definedName>
   </definedNames>
@@ -64,12 +64,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -111,6 +111,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -5848,7 +5852,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>每一行只对应一张 Astro 图片。请先打开“待人工复核 (56)”工作表；此处的图片在 WordPress 导出中没有精确文件名匹配，不能声称继承了旧站 alt。</t>
+          <t>每一行只对应一张 Astro 图片。请先打开“视觉识别补充 alt (56)”工作表；这些图片在 WordPress 导出中没有精确文件名匹配，但已逐张进行本地图片视觉识别并预填可用英文 alt。</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5900,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>“当前建议 alt”显示旧站有效 alt 或当前安全兜底；请把你确认后的版本填写在“你的最终 alt”。</t>
+          <t>“当前建议 alt”与“你的最终 alt”已预填 WordPress 原 alt 或视觉识别 alt。仅当你希望改写时再修改“你的最终 alt”。</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5912,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>请选择：保留 WordPress 原 alt、改用你的最终 alt、装饰性图片 alt=""、或待进一步确认。</t>
+          <t>请选择：保留 WordPress 原 alt、采用视觉识别 alt、改用你的最终 alt、装饰性图片 alt=""、或待进一步确认。</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5969,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
+          <t>已通过视觉识别补充 alt</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -6106,7 +6110,8 @@
 src/pages/lumina-slate.astro
 src/pages/resources/downloads.astro
 src/pages/resources/knowledge-base/what-is-solar-roof.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -6121,17 +6126,29 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Black Lumina Slate active solar roof tile with rear connection cables on a white background.</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Black Lumina Slate active solar roof tile with rear connection cables on a white background.</t>
+        </is>
+      </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="84" customHeight="1">
       <c r="A3" s="5" t="n">
@@ -6150,7 +6167,8 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -6165,17 +6183,29 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Dark textured aluminum valley flashing for a Lumina Slate solar roof.</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Dark textured aluminum valley flashing for a Lumina Slate solar roof.</t>
+        </is>
+      </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="84" customHeight="1">
       <c r="A4" s="5" t="n">
@@ -6195,7 +6225,8 @@
       <c r="E4" s="5" t="inlineStr">
         <is>
           <t>src/pages/resources/knowledge-base/what-is-solar-roof.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -6210,17 +6241,29 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Dark metal eaves starter and drip-edge trim for a Lumina Slate solar roof.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Dark metal eaves starter and drip-edge trim for a Lumina Slate solar roof.</t>
+        </is>
+      </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -6239,7 +6282,8 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -6254,17 +6298,29 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Flexible black flashing roll with protective backing for waterproof solar roof junctions.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Flexible black flashing roll with protective backing for waterproof solar roof junctions.</t>
+        </is>
+      </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="5" t="n">
@@ -6284,7 +6340,8 @@
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>src/pages/resources/knowledge-base/what-is-solar-roof.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -6299,17 +6356,29 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Cuttable black inactive half tile for fitting a Lumina Slate solar roof layout.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Cuttable black inactive half tile for fitting a Lumina Slate solar roof layout.</t>
+        </is>
+      </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="84" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -6328,7 +6397,8 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -6343,17 +6413,29 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Black inactive half tile for completing a Lumina Slate solar roof layout.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Black inactive half tile for completing a Lumina Slate solar roof layout.</t>
+        </is>
+      </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L7" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="84" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -6372,7 +6454,8 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -6387,17 +6470,29 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Black inactive quarter tile for completing a Lumina Slate solar roof layout.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Black inactive quarter tile for completing a Lumina Slate solar roof layout.</t>
+        </is>
+      </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -6416,7 +6511,8 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -6431,17 +6527,29 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Folded black metal rake tile for finishing the sloping edge of a solar roof.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Folded black metal rake tile for finishing the sloping edge of a solar roof.</t>
+        </is>
+      </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="84" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -6460,7 +6568,8 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -6475,17 +6584,29 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Galvanized metal ridge support bracket with mounting holes for a solar roof ridge.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Galvanized metal ridge support bracket with mounting holes for a solar roof ridge.</t>
+        </is>
+      </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="84" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -6506,7 +6627,8 @@
         <is>
           <t>src/pages/about.astro
 src/pages/resources/knowledge-base/what-is-solar-roof.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -6521,17 +6643,29 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Black metal ridge tile for capping the peak of a Lumina Slate solar roof.</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Black metal ridge tile for capping the peak of a Lumina Slate solar roof.</t>
+        </is>
+      </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="84" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -6550,7 +6684,8 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -6565,17 +6700,29 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Ventilated ridge roll with metal mesh and black sealing strip for a solar roof.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Ventilated ridge roll with metal mesh and black sealing strip for a solar roof.</t>
+        </is>
+      </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="84" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -6595,7 +6742,8 @@
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>src/pages/resources/knowledge-base/what-is-solar-roof.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -6610,17 +6758,29 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Narrow black vertical flashing strip for sealing a Lumina Slate solar roof transition.</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Narrow black vertical flashing strip for sealing a Lumina Slate solar roof transition.</t>
+        </is>
+      </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L13" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="84" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -6639,7 +6799,8 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -6654,17 +6815,29 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Pair of black metal wind-uplift clips for securing Lumina Slate roof tiles.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Pair of black metal wind-uplift clips for securing Lumina Slate roof tiles.</t>
+        </is>
+      </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="84" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -6683,7 +6856,8 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -6698,17 +6872,29 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Black butyl sealant tape roll with foil backing for solar roof waterproofing.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Black butyl sealant tape roll with foil backing for solar roof waterproofing.</t>
+        </is>
+      </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L15" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="84" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -6727,7 +6913,8 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -6742,17 +6929,29 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Reflective foil radiant barrier sheet for use beneath a solar roof assembly.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Reflective foil radiant barrier sheet for use beneath a solar roof assembly.</t>
+        </is>
+      </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="84" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -6772,7 +6971,8 @@
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>src/pages/about.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -6787,17 +6987,29 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Pair of black MC4 connectors for photovoltaic cable connections in a solar roof.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Pair of black MC4 connectors for photovoltaic cable connections in a solar roof.</t>
+        </is>
+      </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L17" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -6816,7 +7028,8 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -6831,17 +7044,29 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Stacked timber roof battens for supporting a solar roof installation.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Stacked timber roof battens for supporting a solar roof installation.</t>
+        </is>
+      </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="84" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -6861,7 +7086,8 @@
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>src/pages/resources/knowledge-base/what-is-solar-roof.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -6876,17 +7102,29 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Black waterproof roofing membrane roll for use beneath solar roof components.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Black waterproof roofing membrane roll for use beneath solar roof components.</t>
+        </is>
+      </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="84" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -6906,7 +7144,8 @@
       <c r="E20" s="5" t="inlineStr">
         <is>
           <t>src/pages/resources/downloads.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -6921,17 +7160,29 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Black Storm Guard active solar roof sheet on a white background.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Black Storm Guard active solar roof sheet on a white background.</t>
+        </is>
+      </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="84" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -6950,7 +7201,8 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -6965,17 +7217,29 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Metal mounting fastener for securing a Storm Guard solar roof sheet.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Metal mounting fastener for securing a Storm Guard solar roof sheet.</t>
+        </is>
+      </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="84" customHeight="1">
       <c r="A22" s="5" t="n">
@@ -6994,7 +7258,8 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -7009,17 +7274,29 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Black metal eaves starter and drip-edge strips for a Storm Guard solar roof.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Black metal eaves starter and drip-edge strips for a Storm Guard solar roof.</t>
+        </is>
+      </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="84" customHeight="1">
       <c r="A23" s="5" t="n">
@@ -7038,7 +7315,8 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -7053,17 +7331,29 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Black folded metal flashing boards for Storm Guard solar roof transitions.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Black folded metal flashing boards for Storm Guard solar roof transitions.</t>
+        </is>
+      </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="84" customHeight="1">
       <c r="A24" s="5" t="n">
@@ -7082,7 +7372,8 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -7097,17 +7388,29 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr"/>
-      <c r="J24" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Black metal gable trim panels for finishing a Storm Guard solar roof edge.</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Black metal gable trim panels for finishing a Storm Guard solar roof edge.</t>
+        </is>
+      </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="84" customHeight="1">
       <c r="A25" s="5" t="n">
@@ -7126,7 +7429,8 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -7141,17 +7445,29 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Black metal gutter board with mounting flange for a Storm Guard solar roof.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Black metal gutter board with mounting flange for a Storm Guard solar roof.</t>
+        </is>
+      </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L25" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="84" customHeight="1">
       <c r="A26" s="5" t="n">
@@ -7171,7 +7487,8 @@
       <c r="E26" s="5" t="inlineStr">
         <is>
           <t>src/pages/about.astro
-src/data/componentAssets.ts</t>
+src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -7186,17 +7503,29 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr"/>
-      <c r="J26" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Black non-active metal sheet matching the finish of a Storm Guard solar roof.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Black non-active metal sheet matching the finish of a Storm Guard solar roof.</t>
+        </is>
+      </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="84" customHeight="1">
       <c r="A27" s="5" t="n">
@@ -7215,7 +7544,8 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>src/data/componentAssets.ts</t>
+          <t>src/data/componentAssets.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -7230,17 +7560,29 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Black metal ridge cap assembly for the peak of a Storm Guard solar roof.</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Black metal ridge cap assembly for the peak of a Storm Guard solar roof.</t>
+        </is>
+      </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L27" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="84" customHeight="1">
       <c r="A28" s="5" t="n">
@@ -7259,7 +7601,8 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -7274,17 +7617,29 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Palletized cartons wrapped for storage in a Sunlit warehouse aisle.</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Palletized cartons wrapped for storage in a Sunlit warehouse aisle.</t>
+        </is>
+      </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="84" customHeight="1">
       <c r="A29" s="5" t="n">
@@ -7303,7 +7658,8 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -7318,17 +7674,29 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Palletized inventory stored inside a clean Sunlit warehouse.</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Palletized inventory stored inside a clean Sunlit warehouse.</t>
+        </is>
+      </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L29" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="84" customHeight="1">
       <c r="A30" s="5" t="n">
@@ -7347,7 +7715,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -7362,17 +7730,29 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Exterior view of a warehouse building with loading bays for product dispatch.</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Exterior view of a warehouse building with loading bays for product dispatch.</t>
+        </is>
+      </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="84" customHeight="1">
       <c r="A31" s="5" t="n">
@@ -7391,7 +7771,8 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -7406,17 +7787,29 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Exterior of a photovoltaic building materials laboratory and product showroom.</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>Exterior of a photovoltaic building materials laboratory and product showroom.</t>
+        </is>
+      </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L31" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="84" customHeight="1">
       <c r="A32" s="5" t="n">
@@ -7435,7 +7828,8 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -7450,17 +7844,29 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr"/>
-      <c r="J32" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Factory showroom model demonstrating photovoltaic building applications.</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>Factory showroom model demonstrating photovoltaic building applications.</t>
+        </is>
+      </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L32" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="84" customHeight="1">
       <c r="A33" s="5" t="n">
@@ -7479,7 +7885,8 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -7494,17 +7901,29 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Factory showroom wall displaying framed certificates and product samples.</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Factory showroom wall displaying framed certificates and product samples.</t>
+        </is>
+      </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L33" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="84" customHeight="1">
       <c r="A34" s="5" t="n">
@@ -7523,7 +7942,8 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -7538,17 +7958,29 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Product showroom with a model house and photovoltaic building material displays.</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Product showroom with a model house and photovoltaic building material displays.</t>
+        </is>
+      </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L34" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="84" customHeight="1">
       <c r="A35" s="5" t="n">
@@ -7567,7 +7999,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -7582,17 +8014,29 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr"/>
-      <c r="J35" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Installer fastening a Storm Guard solar roof sheet over a timber batten.</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Installer fastening a Storm Guard solar roof sheet over a timber batten.</t>
+        </is>
+      </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L35" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="84" customHeight="1">
       <c r="A36" s="5" t="n">
@@ -7611,7 +8055,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -7626,17 +8070,29 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr"/>
-      <c r="J36" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Close-up of a metal fastening bracket fixed to a timber batten beside a solar roof sheet.</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>Close-up of a metal fastening bracket fixed to a timber batten beside a solar roof sheet.</t>
+        </is>
+      </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L36" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="84" customHeight="1">
       <c r="A37" s="5" t="n">
@@ -7655,7 +8111,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -7670,17 +8126,29 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr"/>
-      <c r="J37" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Close-up of a metal mounting clip fixed to a timber support for a solar roof sheet.</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Close-up of a metal mounting clip fixed to a timber support for a solar roof sheet.</t>
+        </is>
+      </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L37" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="84" customHeight="1">
       <c r="A38" s="5" t="n">
@@ -7699,7 +8167,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -7714,17 +8182,29 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr"/>
-      <c r="J38" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Indoor demonstration model showing partially assembled Storm Guard metal solar roof sheets.</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>Indoor demonstration model showing partially assembled Storm Guard metal solar roof sheets.</t>
+        </is>
+      </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L38" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="84" customHeight="1">
       <c r="A39" s="5" t="n">
@@ -7743,7 +8223,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -7758,17 +8238,29 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr"/>
-      <c r="J39" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Timber battens arranged across a roof during BIPV solar roof mounting preparation in Beijing.</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>Timber battens arranged across a roof during BIPV solar roof mounting preparation in Beijing.</t>
+        </is>
+      </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L39" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="84" customHeight="1">
       <c r="A40" s="5" t="n">
@@ -7787,7 +8279,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -7802,17 +8294,29 @@
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr"/>
-      <c r="J40" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Dark solar roof tiles installed on a villa beside neighboring residential roofs in Beijing.</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>Dark solar roof tiles installed on a villa beside neighboring residential roofs in Beijing.</t>
+        </is>
+      </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L40" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="84" customHeight="1">
       <c r="A41" s="5" t="n">
@@ -7831,7 +8335,8 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -7846,17 +8351,29 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr"/>
-      <c r="J41" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>High-angle view of a staggered dark solar tile layout on a Beijing villa roof.</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>High-angle view of a staggered dark solar tile layout on a Beijing villa roof.</t>
+        </is>
+      </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L41" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="84" customHeight="1">
       <c r="A42" s="5" t="n">
@@ -7875,7 +8392,8 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -7890,17 +8408,29 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr"/>
-      <c r="J42" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Dark Lumina Slate solar roof tiles integrated beside traditional grey roof tiles on a villa.</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>Dark Lumina Slate solar roof tiles integrated beside traditional grey roof tiles on a villa.</t>
+        </is>
+      </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L42" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="84" customHeight="1">
       <c r="A43" s="5" t="n">
@@ -7919,7 +8449,8 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -7934,17 +8465,29 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Red electrical cables laid across dark solar roof tiles during a residential installation.</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>Red electrical cables laid across dark solar roof tiles during a residential installation.</t>
+        </is>
+      </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L43" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="84" customHeight="1">
       <c r="A44" s="5" t="n">
@@ -7963,7 +8506,8 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -7978,17 +8522,29 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr"/>
-      <c r="J44" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Dark solar roof tiles with cable connections during a residential BIPV installation.</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>Dark solar roof tiles with cable connections during a residential BIPV installation.</t>
+        </is>
+      </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L44" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="84" customHeight="1">
       <c r="A45" s="5" t="n">
@@ -8007,7 +8563,8 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -8022,17 +8579,29 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr"/>
-      <c r="J45" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Completed Nanjing villa with a dark integrated solar roof under a blue sky.</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Completed Nanjing villa with a dark integrated solar roof under a blue sky.</t>
+        </is>
+      </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L45" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="84" customHeight="1">
       <c r="A46" s="5" t="n">
@@ -8051,7 +8620,8 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
@@ -8066,17 +8636,29 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I46" s="5" t="inlineStr"/>
-      <c r="J46" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Front view of a Nanjing residential villa with a dark integrated solar roof.</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Front view of a Nanjing residential villa with a dark integrated solar roof.</t>
+        </is>
+      </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L46" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="84" customHeight="1">
       <c r="A47" s="5" t="n">
@@ -8095,7 +8677,8 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -8110,17 +8693,29 @@
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I47" s="5" t="inlineStr"/>
-      <c r="J47" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Worker installing dark solar roof tiles on a public facility roof.</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Worker installing dark solar roof tiles on a public facility roof.</t>
+        </is>
+      </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L47" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="84" customHeight="1">
       <c r="A48" s="5" t="n">
@@ -8139,7 +8734,8 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>src/data/projects.ts</t>
+          <t>src/data/projects.ts
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -8154,17 +8750,29 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr"/>
-      <c r="J48" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Shanghai villa with a dark solar roof installed as a residential upgrade.</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>Shanghai villa with a dark solar roof installed as a residential upgrade.</t>
+        </is>
+      </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L48" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="84" customHeight="1">
       <c r="A49" s="5" t="n">
@@ -8183,7 +8791,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -8198,17 +8806,29 @@
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr"/>
-      <c r="J49" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Aerial view of a large gymnasium roof under BIPV solar roof installation in the United States.</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Aerial view of a large gymnasium roof under BIPV solar roof installation in the United States.</t>
+        </is>
+      </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L49" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="84" customHeight="1">
       <c r="A50" s="5" t="n">
@@ -8227,7 +8847,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
@@ -8242,17 +8862,29 @@
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I50" s="5" t="inlineStr"/>
-      <c r="J50" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Timber battens and roof membrane prepared for a gymnasium solar roof installation in the United States.</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Timber battens and roof membrane prepared for a gymnasium solar roof installation in the United States.</t>
+        </is>
+      </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L50" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="84" customHeight="1">
       <c r="A51" s="5" t="n">
@@ -8271,7 +8903,8 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -8286,17 +8919,29 @@
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr"/>
-      <c r="J51" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Rows of black solar roof sheets stacked on pallets in a factory warehouse.</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Rows of black solar roof sheets stacked on pallets in a factory warehouse.</t>
+        </is>
+      </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L51" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="84" customHeight="1">
       <c r="A52" s="5" t="n">
@@ -8315,7 +8960,8 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -8330,17 +8976,29 @@
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr"/>
-      <c r="J52" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Stacked black solar roof sheets on a wooden pallet in a factory.</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>Stacked black solar roof sheets on a wooden pallet in a factory.</t>
+        </is>
+      </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L52" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="84" customHeight="1">
       <c r="A53" s="5" t="n">
@@ -8359,7 +9017,8 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>src/pages/about.astro</t>
+          <t>src/pages/about.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -8374,17 +9033,29 @@
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr"/>
-      <c r="J53" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Wooden shipping crate packed for transport of solar roof components.</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>Wooden shipping crate packed for transport of solar roof components.</t>
+        </is>
+      </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L53" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="84" customHeight="1">
       <c r="A54" s="5" t="n">
@@ -8404,7 +9075,8 @@
       <c r="E54" s="5" t="inlineStr">
         <is>
           <t>src/pages/about.astro
-src/pages/index.astro</t>
+src/pages/index.astro
+src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -8419,17 +9091,29 @@
       </c>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I54" s="5" t="inlineStr"/>
-      <c r="J54" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Line of wooden pallets loaded with packaged solar roof products in a factory corridor.</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>Line of wooden pallets loaded with packaged solar roof products in a factory corridor.</t>
+        </is>
+      </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L54" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="84" customHeight="1">
       <c r="A55" s="5" t="n">
@@ -8448,7 +9132,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -8463,17 +9147,29 @@
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I55" s="5" t="inlineStr"/>
-      <c r="J55" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>Factory staff inspecting a black solar roof sheet at a quality-control workstation.</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Factory staff inspecting a black solar roof sheet at a quality-control workstation.</t>
+        </is>
+      </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L55" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="84" customHeight="1">
       <c r="A56" s="5" t="n">
@@ -8492,7 +9188,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -8507,17 +9203,29 @@
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr"/>
-      <c r="J56" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Black solar roof sheets stacked on a pallet with protective white spacers.</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>Black solar roof sheets stacked on a pallet with protective white spacers.</t>
+        </is>
+      </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L56" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="84" customHeight="1">
       <c r="A57" s="5" t="n">
@@ -8536,7 +9244,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>未检测到直接引用</t>
+          <t>src/data/imageAltManifest.ts</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -8551,17 +9259,29 @@
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>需人工复核：无精确 WordPress 文件匹配</t>
-        </is>
-      </c>
-      <c r="I57" s="5" t="inlineStr"/>
-      <c r="J57" s="5" t="inlineStr"/>
+          <t>无精确 WordPress 匹配；已完成本地视觉识别</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Shipping label attached to a shrink-wrapped pallet of solar roof products.</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>Shipping label attached to a shrink-wrapped pallet of solar roof products.</t>
+        </is>
+      </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>待进一步确认</t>
-        </is>
-      </c>
-      <c r="L57" s="5" t="inlineStr"/>
+          <t>采用视觉识别 alt</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>视觉识别来源：docs/visual-reviewed-image-alt.json</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L57"/>
@@ -8572,7 +9292,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="K2:K57 K2:K139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"保留 WordPress 原 alt,改用你的最终 alt,装饰性图片 alt="",待进一步确认"</formula1>
+      <formula1>"保留 WordPress 原 alt,采用视觉识别 alt,改用你的最终 alt,装饰性图片 alt="",待进一步确认"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15995,7 +16715,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="K2:K57 K2:K139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"保留 WordPress 原 alt,改用你的最终 alt,装饰性图片 alt="",待进一步确认"</formula1>
+      <formula1>"保留 WordPress 原 alt,采用视觉识别 alt,改用你的最终 alt,装饰性图片 alt="",待进一步确认"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16089,53 +16809,53 @@
       </c>
     </row>
     <row r="2" ht="84" customHeight="1">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>/images/articles/how-to-install-solar-roof/cover.png</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>public/images/articles/how-to-install-solar-roof/cover.png</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>src/data/articleMedia.ts
 src/content/articles/how-to-install-solar-roof.md</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>https://www.sunlitsolarroof.com/wp-content/uploads/2025/10/news.png</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>旧站 alt 为空/泛化：需人工复核</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>Article cover image for How to Install a Solar Roof: A No-Nonsense Guide for Builders</t>
         </is>
       </c>
-      <c r="J2" s="5" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>Article cover image for How to Install a Solar Roof: A No-Nonsense Guide for Builders</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>待进一步确认</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>文章：how-to-install-solar-roof；角色：封面图；章节：封面</t>
         </is>
@@ -16199,171 +16919,171 @@
       </c>
     </row>
     <row r="4" ht="84" customHeight="1">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="B4" s="10" t="n"/>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>/images/articles/what-is-a-solar-roof/cover.webp</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>public/images/articles/what-is-a-solar-roof/cover.webp</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>src/data/articleMedia.ts
 src/content/articles/what-is-a-solar-roof.md</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>https://www.sunlitsolarroof.com/wp-content/uploads/2025/12/Roof-tiles-3-scaled.webp</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>Roof tiles 3</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>旧站 alt 为空/泛化：需人工复核</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Article cover image for What is a Solar Roof? And Why 2026 is the Year to Make Your Move</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>Article cover image for What is a Solar Roof? And Why 2026 is the Year to Make Your Move</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>待进一步确认</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>文章：what-is-a-solar-roof；角色：封面图；章节：封面</t>
         </is>
       </c>
     </row>
     <row r="5" ht="84" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>/images/articles/solar-roof-roi-for-developers/cover.webp</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>public/images/articles/solar-roof-roi-for-developers/cover.webp</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>src/data/articleMedia.ts
 src/content/articles/solar-roof-roi-for-developers.md</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>https://www.sunlitsolarroof.com/wp-content/uploads/2025/10/solutions-banner.webp</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>solutions banner</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>旧站 alt 为空/泛化：需人工复核</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>Article cover image for Why Developers Are Doing the Math Wrong on Solar Roofs</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr">
         <is>
           <t>Article cover image for Why Developers Are Doing the Math Wrong on Solar Roofs</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>待进一步确认</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>文章：solar-roof-roi-for-developers；角色：封面图；章节：封面</t>
         </is>
       </c>
     </row>
     <row r="6" ht="84" customHeight="1">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>/images/articles/solar-roof-case-study/cover.png</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>public/images/articles/solar-roof-case-study/cover.png</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>src/data/articleMedia.ts
 src/content/articles/solar-roof-case-study.md</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>https://www.sunlitsolarroof.com/wp-content/uploads/2025/10/about-sunlit.png</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>about sunlit</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>旧站 alt 为空/泛化：需人工复核</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Article cover image for A Real Case Study: Building a Solar Roof Across the Ocean</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>Article cover image for A Real Case Study: Building a Solar Roof Across the Ocean</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>待进一步确认</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>文章：solar-roof-case-study；角色：封面图；章节：封面</t>
         </is>
@@ -16484,53 +17204,53 @@
       </c>
     </row>
     <row r="9" ht="84" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>/images/articles/lumina-slate-story/cover.jpg</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>public/images/articles/lumina-slate-story/cover.jpg</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>src/data/articleMedia.ts
 src/content/articles/lumina-slate-story.md</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>https://www.sunlitsolarroof.com/wp-content/uploads/2026/04/907250b58e09c6f80c09777050900289.jpg</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>旧站 alt 为空/泛化：需人工复核</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>Article cover image for The Story Behind Lumina Slate: Building a Better Solar Roof</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="9" t="inlineStr">
         <is>
           <t>Article cover image for The Story Behind Lumina Slate: Building a Better Solar Roof</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>待进一步确认</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
         <is>
           <t>文章：lumina-slate-story；角色：封面图；章节：封面</t>
         </is>
@@ -16594,57 +17314,57 @@
       </c>
     </row>
     <row r="11" ht="84" customHeight="1">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>/images/articles/solar-roofing-business-model/cover.jpg</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>public/images/articles/solar-roofing-business-model/cover.jpg</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>src/data/articleMedia.ts
 src/content/articles/solar-roofing-business-model.md</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>https://www.sunlitsolarroof.com/wp-content/uploads/2025/12/home-scaled.jpg</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>旧站 alt 为空/泛化：需人工复核</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>Article cover image for The "IKEA Model" of Solar Roofing: Who We Work With (And Why We Say No)</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="9" t="inlineStr">
         <is>
           <t>Article cover image for The "IKEA Model" of Solar Roofing: Who We Work With (And Why We Say No)</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>待进一步确认</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>文章：solar-roofing-business-model；角色：封面图；章节：封面</t>
         </is>
@@ -17115,7 +17835,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="K2:K57 K2:K139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"保留 WordPress 原 alt,改用你的最终 alt,装饰性图片 alt="",待进一步确认"</formula1>
+      <formula1>"保留 WordPress 原 alt,采用视觉识别 alt,改用你的最终 alt,装饰性图片 alt="",待进一步确认"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>